<commit_message>
Add quarterly UW market rents, record model refresh
</commit_message>
<xml_diff>
--- a/knowledge/exhibits/Rent_Chart_Data.xlsx
+++ b/knowledge/exhibits/Rent_Chart_Data.xlsx
@@ -122,16 +122,16 @@
     <t xml:space="preserve">Seasons T90 effective (mix-wtd)</t>
   </si>
   <si>
-    <t xml:space="preserve">Seasons UW mkt rent (yr avg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seasons L5 / UW entry</t>
+    <t xml:space="preserve">Seasons UW market rent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seasons L5 executed (8/4/26)</t>
   </si>
   <si>
     <t xml:space="preserve">Prelude T90 (mix-wtd)</t>
   </si>
   <si>
-    <t xml:space="preserve">Prelude UW rent/occ (yr avg)</t>
+    <t xml:space="preserve">Prelude UW market rent</t>
   </si>
   <si>
     <t xml:space="preserve">Prelude actual in-place</t>
@@ -140,7 +140,7 @@
     <t xml:space="preserve">Prelude L5 (8/13/26)</t>
   </si>
   <si>
-    <t xml:space="preserve">UW market rents are ANNUAL AVERAGES, plotted at UW-year midpoints: Seasons Y1 (Nov-26..Oct-27) avg $1,885 sits at Apr-27, then +4/4/3.5/3.5/3% steps; Prelude UW = calendar-year averages at Jul-1. Seasons L5 marker 8/4/26 = executed new-lease spot. Actuals: potential rent net LTL /280 from accrual statement.</t>
+    <t xml:space="preserve">UW market rents are period AVERAGES: quarterly (calendar quarters, plotted mid-quarter) through Y1, annual (plotted at UW-year midpoints) beyond. Seasons = updated model Rent &amp; Occ Data row 5: TMG Y1 = 4Q26-3Q27 avg $1,933.28, then +4/4/3.5/3.5/3%. Prelude = Market Rent Summary row 11 (Q4-25 anchor + TMG Y1 calendar-2026 quarters, avg $1,729.6), then CF Market Rent /280/12. Seasons L5 marker 8/4/26 = executed new-lease spot. Actuals: potential rent net LTL /280 from accrual statement.</t>
   </si>
   <si>
     <t xml:space="preserve">Floorplan Mapped</t>
@@ -4908,7 +4908,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:K53"/>
+  <dimension ref="B2:K57"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -5234,194 +5234,200 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="16" t="n">
+        <v>45976</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>1693</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="16" t="n">
         <v>45991</v>
       </c>
-      <c r="C22" s="17" t="n">
+      <c r="C23" s="17" t="n">
         <f aca="false">T90_Monthly!U16</f>
         <v>1679.63697089947</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D23" s="17" t="n">
         <f aca="false">T90_Monthly!U29</f>
         <v>1419.62533068783</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="G23" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!U37)</f>
         <v>1693.68112244898</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="16" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="16" t="n">
         <v>46022</v>
       </c>
-      <c r="C23" s="17" t="n">
+      <c r="C24" s="17" t="n">
         <f aca="false">T90_Monthly!V16</f>
         <v>1676.65393518519</v>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D24" s="17" t="n">
         <f aca="false">T90_Monthly!V29</f>
         <v>1423.47106481482</v>
       </c>
-      <c r="G23" s="17" t="n">
+      <c r="G24" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!V37)</f>
         <v>1703.96031746032</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="16" t="n">
-        <v>46037</v>
-      </c>
-      <c r="I24" s="10" t="n">
-        <v>1668</v>
-      </c>
-    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="16" t="n">
+        <v>46037</v>
+      </c>
+      <c r="I25" s="10" t="n">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="16" t="n">
         <v>46053</v>
       </c>
-      <c r="C25" s="17" t="n">
+      <c r="C26" s="17" t="n">
         <f aca="false">T90_Monthly!W16</f>
         <v>1698.00978535354</v>
       </c>
-      <c r="D25" s="17" t="n">
+      <c r="D26" s="17" t="n">
         <f aca="false">T90_Monthly!W29</f>
         <v>1476.7086489899</v>
       </c>
-      <c r="G25" s="17" t="n">
+      <c r="G26" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!W37)</f>
         <v>1714.91326530612</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="16" t="n">
-        <v>46068</v>
-      </c>
-      <c r="I26" s="10" t="n">
-        <v>1670</v>
-      </c>
-    </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="16" t="n">
+        <v>46068</v>
+      </c>
+      <c r="H27" s="10" t="n">
+        <v>1712.3</v>
+      </c>
+      <c r="I27" s="10" t="n">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="16" t="n">
         <v>46081</v>
       </c>
-      <c r="C27" s="17" t="n">
+      <c r="C28" s="17" t="n">
         <f aca="false">T90_Monthly!X16</f>
         <v>1678.38017676768</v>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D28" s="17" t="n">
         <f aca="false">T90_Monthly!X29</f>
         <v>1516.18080808081</v>
       </c>
-      <c r="G27" s="17" t="n">
+      <c r="G28" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!X37)</f>
         <v>1695.69285714286</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="16" t="n">
-        <v>46096</v>
-      </c>
-      <c r="I28" s="10" t="n">
-        <v>1672</v>
-      </c>
-    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="16" t="n">
+        <v>46096</v>
+      </c>
+      <c r="I29" s="10" t="n">
+        <v>1672</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="16" t="n">
         <v>46112</v>
       </c>
-      <c r="C29" s="17" t="n">
+      <c r="C30" s="17" t="n">
         <f aca="false">T90_Monthly!Y16</f>
         <v>1722.68074770928</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D30" s="17" t="n">
         <f aca="false">T90_Monthly!Y29</f>
         <v>1580.24360463793</v>
       </c>
-      <c r="G29" s="17" t="n">
+      <c r="G30" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!Y37)</f>
         <v>1629.02380952381</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="16" t="n">
-        <v>46127</v>
-      </c>
-      <c r="I30" s="10" t="n">
-        <v>1675</v>
-      </c>
-    </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="16" t="n">
+        <v>46127</v>
+      </c>
+      <c r="I31" s="10" t="n">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="16" t="n">
         <v>46142</v>
       </c>
-      <c r="C31" s="17" t="n">
+      <c r="C32" s="17" t="n">
         <f aca="false">T90_Monthly!Z16</f>
         <v>1763.60901559454</v>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D32" s="17" t="n">
         <f aca="false">T90_Monthly!Z29</f>
         <v>1627.761024088</v>
       </c>
-      <c r="G31" s="17" t="n">
+      <c r="G32" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!Z37)</f>
         <v>1651.61961951447</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="16" t="n">
-        <v>46157</v>
-      </c>
-      <c r="I32" s="10" t="n">
-        <v>1675</v>
-      </c>
-    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="16" t="n">
+        <v>46157</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <v>1732.2</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="16" t="n">
         <v>46173</v>
       </c>
-      <c r="C33" s="17" t="n">
+      <c r="C34" s="17" t="n">
         <f aca="false">T90_Monthly!AA16</f>
         <v>1836.23011525512</v>
       </c>
-      <c r="D33" s="17" t="n">
+      <c r="D34" s="17" t="n">
         <f aca="false">T90_Monthly!AA29</f>
         <v>1723.50387852888</v>
       </c>
-      <c r="G33" s="17" t="n">
+      <c r="G34" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!AA37)</f>
         <v>1675.61171579743</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="16" t="n">
-        <v>46188</v>
-      </c>
-      <c r="I34" s="10" t="n">
-        <v>1682</v>
-      </c>
-    </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="16" t="n">
+        <v>46188</v>
+      </c>
+      <c r="I35" s="10" t="n">
+        <v>1682</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="16" t="n">
         <v>46203</v>
       </c>
-      <c r="C35" s="17" t="n">
+      <c r="C36" s="17" t="n">
         <f aca="false">T90_Monthly!AB16</f>
         <v>1913.6579423436</v>
       </c>
-      <c r="D35" s="17" t="n">
+      <c r="D36" s="17" t="n">
         <f aca="false">T90_Monthly!AB29</f>
         <v>1858.3439056178</v>
       </c>
-      <c r="G35" s="17" t="n">
+      <c r="G36" s="17" t="n">
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!AB37)</f>
         <v>1707.15951933405</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="16" t="n">
-        <v>46204</v>
-      </c>
-      <c r="H36" s="10" t="n">
-        <v>1668</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5481,113 +5487,148 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="16" t="n">
-        <v>46507</v>
-      </c>
-      <c r="E41" s="10" t="n">
-        <v>1885</v>
+        <v>46249</v>
+      </c>
+      <c r="H41" s="10" t="n">
+        <v>1745.5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="16" t="n">
-        <v>46569</v>
+        <v>46341</v>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>1902.2</v>
       </c>
       <c r="H42" s="10" t="n">
-        <v>1745</v>
+        <v>1728.5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="16" t="n">
-        <v>46873</v>
+        <v>46433</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>1960</v>
+        <v>1923.1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="16" t="n">
-        <v>46935</v>
-      </c>
-      <c r="H44" s="10" t="n">
-        <v>1808</v>
+        <v>46522</v>
+      </c>
+      <c r="E44" s="10" t="n">
+        <v>1946.2</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B45" s="16" t="n">
-        <v>47238</v>
-      </c>
-      <c r="E45" s="10" t="n">
-        <v>2038</v>
+        <v>46569</v>
+      </c>
+      <c r="H45" s="10" t="n">
+        <v>1775.8</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="16" t="n">
-        <v>47300</v>
-      </c>
-      <c r="H46" s="10" t="n">
-        <v>1883</v>
+        <v>46614</v>
+      </c>
+      <c r="E46" s="10" t="n">
+        <v>1961.7</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B47" s="16" t="n">
-        <v>47603</v>
+        <v>46873</v>
       </c>
       <c r="E47" s="10" t="n">
-        <v>2110</v>
+        <v>2010.6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B48" s="16" t="n">
-        <v>47665</v>
+        <v>46935</v>
       </c>
       <c r="H48" s="10" t="n">
-        <v>1952</v>
+        <v>1838.2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B49" s="16" t="n">
-        <v>47968</v>
+        <v>47238</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>2184</v>
+        <v>2091</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="16" t="n">
+        <v>47300</v>
+      </c>
+      <c r="H50" s="10" t="n">
+        <v>1906.7</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B51" s="16" t="n">
+        <v>47603</v>
+      </c>
+      <c r="E51" s="10" t="n">
+        <v>2164.2</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="16" t="n">
+        <v>47665</v>
+      </c>
+      <c r="H52" s="10" t="n">
+        <v>1976.5</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="16" t="n">
+        <v>47968</v>
+      </c>
+      <c r="E53" s="10" t="n">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="16" t="n">
         <v>48334</v>
       </c>
-      <c r="E50" s="10" t="n">
-        <v>2249</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="2" t="s">
+      <c r="E54" s="10" t="n">
+        <v>2307.2</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C52" s="2"/>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
-      <c r="I52" s="2"/>
-      <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+      <c r="G56" s="2"/>
+      <c r="H56" s="2"/>
+      <c r="I56" s="2"/>
+      <c r="J56" s="2"/>
+      <c r="K56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+      <c r="G57" s="2"/>
+      <c r="H57" s="2"/>
+      <c r="I57" s="2"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B52:K53"/>
+    <mergeCell ref="B56:K57"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Quarterly UW points on month-end dates, add acquisition L5 marker
</commit_message>
<xml_diff>
--- a/knowledge/exhibits/Rent_Chart_Data.xlsx
+++ b/knowledge/exhibits/Rent_Chart_Data.xlsx
@@ -137,10 +137,10 @@
     <t xml:space="preserve">Prelude actual in-place</t>
   </si>
   <si>
-    <t xml:space="preserve">Prelude L5 (8/13/26)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UW market rents are period AVERAGES: quarterly (calendar quarters, plotted mid-quarter) through Y1, annual (plotted at UW-year midpoints) beyond. Seasons = updated model Rent &amp; Occ Data row 5: TMG Y1 = 4Q26-3Q27 avg $1,933.28, then +4/4/3.5/3.5/3%. Prelude = Market Rent Summary row 11 (Q4-25 anchor + TMG Y1 calendar-2026 quarters, avg $1,729.6), then CF Market Rent /280/12. Seasons L5 marker 8/4/26 = executed new-lease spot. Actuals: potential rent net LTL /280 from accrual statement.</t>
+    <t xml:space="preserve">Prelude L5 (acq 12/3/25 + 8/13/26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UW market rents are period AVERAGES: quarterly (calendar quarters, plotted mid-quarter) through Y1, annual (plotted at UW-year midpoints) beyond. Seasons = updated model Rent &amp; Occ Data row 5: TMG Y1 = 4Q26-3Q27 avg $1,933.28, then +4/4/3.5/3.5/3%. Prelude = Market Rent Summary row 11 (Q4-25 anchor + TMG Y1 calendar-2026 quarters, avg $1,729.6), then CF Market Rent /280/12. Seasons L5 marker 8/4/26 = executed new-lease spot. Prelude L5 markers: $1,717.5 at acquisition (Market Rent Summary "L5 New" wtd avg, RR 12/3/25) and $1,810.62 current (RR 8/13/26). Actuals: potential rent net LTL /280 from accrual statement.</t>
   </si>
   <si>
     <t xml:space="preserve">Floorplan Mapped</t>
@@ -5234,7 +5234,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="16" t="n">
-        <v>45976</v>
+        <v>45991</v>
+      </c>
+      <c r="C22" s="17" t="n">
+        <f aca="false">T90_Monthly!U16</f>
+        <v>1679.63697089947</v>
+      </c>
+      <c r="D22" s="17" t="n">
+        <f aca="false">T90_Monthly!U29</f>
+        <v>1419.62533068783</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!U37)</f>
+        <v>1693.68112244898</v>
       </c>
       <c r="H22" s="10" t="n">
         <v>1693</v>
@@ -5242,19 +5254,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="16" t="n">
-        <v>45991</v>
-      </c>
-      <c r="C23" s="17" t="n">
-        <f aca="false">T90_Monthly!U16</f>
-        <v>1679.63697089947</v>
-      </c>
-      <c r="D23" s="17" t="n">
-        <f aca="false">T90_Monthly!U29</f>
-        <v>1419.62533068783</v>
-      </c>
-      <c r="G23" s="17" t="n">
-        <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!U37)</f>
-        <v>1693.68112244898</v>
+        <v>45994</v>
+      </c>
+      <c r="J23" s="10" t="n">
+        <v>1717.5</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5303,9 +5306,6 @@
       <c r="B27" s="16" t="n">
         <v>46068</v>
       </c>
-      <c r="H27" s="10" t="n">
-        <v>1712.3</v>
-      </c>
       <c r="I27" s="10" t="n">
         <v>1670</v>
       </c>
@@ -5326,6 +5326,9 @@
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!X37)</f>
         <v>1695.69285714286</v>
       </c>
+      <c r="H28" s="10" t="n">
+        <v>1712.3</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="16" t="n">
@@ -5381,9 +5384,6 @@
       <c r="B33" s="16" t="n">
         <v>46157</v>
       </c>
-      <c r="H33" s="10" t="n">
-        <v>1732.2</v>
-      </c>
       <c r="I33" s="10" t="n">
         <v>1675</v>
       </c>
@@ -5404,6 +5404,9 @@
         <f aca="false">IF(T90_Monthly!$D$38=0,"",T90_Monthly!AA37)</f>
         <v>1675.61171579743</v>
       </c>
+      <c r="H34" s="10" t="n">
+        <v>1732.2</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="16" t="n">
@@ -5487,7 +5490,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="16" t="n">
-        <v>46249</v>
+        <v>46265</v>
       </c>
       <c r="H41" s="10" t="n">
         <v>1745.5</v>
@@ -5495,7 +5498,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="16" t="n">
-        <v>46341</v>
+        <v>46356</v>
       </c>
       <c r="E42" s="10" t="n">
         <v>1902.2</v>
@@ -5506,7 +5509,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="16" t="n">
-        <v>46433</v>
+        <v>46446</v>
       </c>
       <c r="E43" s="10" t="n">
         <v>1923.1</v>
@@ -5514,7 +5517,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="16" t="n">
-        <v>46522</v>
+        <v>46538</v>
       </c>
       <c r="E44" s="10" t="n">
         <v>1946.2</v>
@@ -5530,7 +5533,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B46" s="16" t="n">
-        <v>46614</v>
+        <v>46630</v>
       </c>
       <c r="E46" s="10" t="n">
         <v>1961.7</v>

</xml_diff>

<commit_message>
Add Prelude Y6 UW market rent point
</commit_message>
<xml_diff>
--- a/knowledge/exhibits/Rent_Chart_Data.xlsx
+++ b/knowledge/exhibits/Rent_Chart_Data.xlsx
@@ -5502,7 +5502,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:L57"/>
+  <dimension ref="B2:L58"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -6299,29 +6299,24 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B54" s="16" t="n">
+        <v>48030</v>
+      </c>
+      <c r="I54" s="10" t="n">
+        <v>2045.2</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B55" s="16" t="n">
         <v>48334</v>
       </c>
-      <c r="E54" s="10" t="n">
+      <c r="E55" s="10" t="n">
         <v>2307.2</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="2" t="s">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B57" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-      <c r="G56" s="2"/>
-      <c r="H56" s="2"/>
-      <c r="I56" s="2"/>
-      <c r="J56" s="2"/>
-      <c r="K56" s="2"/>
-      <c r="L56" s="2"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
@@ -6333,9 +6328,22 @@
       <c r="K57" s="2"/>
       <c r="L57" s="2"/>
     </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+      <c r="G58" s="2"/>
+      <c r="H58" s="2"/>
+      <c r="I58" s="2"/>
+      <c r="J58" s="2"/>
+      <c r="K58" s="2"/>
+      <c r="L58" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B56:L57"/>
+    <mergeCell ref="B57:L58"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>